<commit_message>
Update parameter estimates after changing stage 2 baseline categories
</commit_message>
<xml_diff>
--- a/input/reg_RMSE.xlsx
+++ b/input/reg_RMSE.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10222"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/Sonnewald/GitHub/SimPaths/input/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\eii2t\src\SimPaths\input\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9F31421A-A2A9-134E-BAE0-B0FAE2CD5120}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5EE0A200-6B20-407D-A212-F87533098329}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="18980" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="UK" sheetId="1" r:id="rId1"/>
@@ -479,9 +479,9 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:B27"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -489,7 +489,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>5</v>
       </c>
@@ -497,7 +497,7 @@
         <v>0.81857066434101511</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>6</v>
       </c>
@@ -505,7 +505,7 @@
         <v>0.83183050833110173</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>7</v>
       </c>
@@ -513,7 +513,7 @@
         <v>0.52838226151512502</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>8</v>
       </c>
@@ -521,7 +521,7 @@
         <v>0.63794775886311106</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>2</v>
       </c>
@@ -529,7 +529,7 @@
         <v>1.7487317224564645</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>3</v>
       </c>
@@ -537,7 +537,7 @@
         <v>3.7549875108949018</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>4</v>
       </c>
@@ -545,7 +545,7 @@
         <v>6.4764075049781749</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>9</v>
       </c>
@@ -553,7 +553,7 @@
         <v>1.0366118799278699</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>10</v>
       </c>
@@ -561,7 +561,7 @@
         <v>0.85170355381228569</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>11</v>
       </c>
@@ -569,7 +569,7 @@
         <v>1.1480377870969753</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>12</v>
       </c>
@@ -577,95 +577,95 @@
         <v>1.1960390964496237</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>13</v>
       </c>
       <c r="B13">
-        <v>4.460523583140219</v>
-      </c>
-    </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.2">
+        <v>4.4589755398683391</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>14</v>
       </c>
       <c r="B14">
-        <v>4.2529536919897684</v>
-      </c>
-    </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.2">
+        <v>4.2447678638002282</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>15</v>
       </c>
       <c r="B15">
-        <v>3.7382957371324035</v>
-      </c>
-    </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.2">
+        <v>3.7326763899982205</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>16</v>
       </c>
       <c r="B16">
-        <v>2.5977267935063337</v>
-      </c>
-    </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.2">
+        <v>2.5967180465968904</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>17</v>
       </c>
       <c r="B17">
-        <v>2.1895888225015536</v>
-      </c>
-    </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.2">
+        <v>2.1881635338703331</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>18</v>
       </c>
       <c r="B18">
-        <v>7.9661177286442255</v>
-      </c>
-    </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.2">
+        <v>7.9633974319488701</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>19</v>
       </c>
       <c r="B19">
-        <v>7.1714148232921389</v>
-      </c>
-    </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.2">
+        <v>7.1575015721166011</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>20</v>
       </c>
       <c r="B20">
-        <v>6.4840573935244814</v>
-      </c>
-    </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.2">
+        <v>6.4812771229350554</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>21</v>
       </c>
       <c r="B21">
-        <v>7.0657713186475233</v>
-      </c>
-    </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.2">
+        <v>7.053059789425987</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>22</v>
       </c>
       <c r="B22">
-        <v>6.0610553268076588</v>
-      </c>
-    </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.2">
+        <v>6.0356409060988723</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>23</v>
       </c>
       <c r="B23">
-        <v>5.4194767626250133</v>
-      </c>
-    </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.2">
+        <v>5.3999363502151345</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>24</v>
       </c>
@@ -673,7 +673,7 @@
         <v>1.9023687544636687</v>
       </c>
     </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>25</v>
       </c>
@@ -681,7 +681,7 @@
         <v>1.7145370168869383</v>
       </c>
     </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>26</v>
       </c>
@@ -689,7 +689,7 @@
         <v>1.6259752837992298</v>
       </c>
     </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A27" s="1" t="s">
         <v>27</v>
       </c>

</xml_diff>